<commit_message>
feat: implementacion de arquitectura etl sat v2 con procesamiento out-of-core
</commit_message>
<xml_diff>
--- a/Diccionario de Datos SAT.xlsx
+++ b/Diccionario de Datos SAT.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\addominguez\Documents\Bases de Datos SQL\ETL_SAT_V2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8218E687-A86D-4A52-AE62-3241FC66DC40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47ECA28-0F3B-4CE3-A5E9-CE59D11231B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6B9CC223-D15A-45F1-BE59-C46A2CDE5E59}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6B9CC223-D15A-45F1-BE59-C46A2CDE5E59}"/>
   </bookViews>
   <sheets>
     <sheet name="SAT" sheetId="1" r:id="rId1"/>
     <sheet name="SAT-Nómina" sheetId="3" r:id="rId2"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="202">
   <si>
     <t>UUID</t>
   </si>
@@ -319,321 +318,6 @@
     <t>GERG_AECF_1891_Anexo2B-QA</t>
   </si>
   <si>
-    <t>Archivo</t>
-  </si>
-  <si>
-    <t>Filas</t>
-  </si>
-  <si>
-    <t>GERG_AECF_1891_Anexo2B.csv</t>
-  </si>
-  <si>
-    <t>Script DDL: Tabla Maestra (Anexo 1A)</t>
-  </si>
-  <si>
-    <t>CREATE TABLE ANEXO_1A_2025_1S (</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    -- Llave Primaria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [UUID] VARCHAR(36) NOT NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    </t>
-  </si>
-  <si>
-    <t xml:space="preserve">    -- Fechas principales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [FechaEmision] DATETIME NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [FechaCertificacion] DATETIME NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [FechaCancelacion] DATETIME NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    -- Importes Financieros (Alineados a 6 decimales según estándar SAT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [SubTotal] DECIMAL(18,6) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [Descuento] DECIMAL(18,6) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [Total] DECIMAL(18,6) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [TrasladosIVA] DECIMAL(18,6) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [TrasladosIEPS] DECIMAL(18,6) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [TotalImpuestosTrasladados] DECIMAL(18,6) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [RetenidosIVA] DECIMAL(18,6) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [RetenidosISR] DECIMAL(18,6) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [TotalImpuestosRetenidos] DECIMAL(18,6) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    -- Moneda y Tipo de Cambio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [Moneda] VARCHAR(3) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [TipoCambio] DECIMAL(18,6) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    -- Clasificadores del Comprobante</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [TipoDeComprobante] VARCHAR(5) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [MetodoPago] VARCHAR(5) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [FormaPago] VARCHAR(5) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [CondicionesDePago] VARCHAR(MAX) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    -- Datos de los Actores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [EmisorRFC] VARCHAR(15) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [EmisorNombre] VARCHAR(MAX) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [EmisorRegimenFiscal] VARCHAR(5) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [ReceptorRFC] VARCHAR(15) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [ReceptorNombre] VARCHAR(MAX) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    -- Datos de Control Interno del Emisor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [Serie] VARCHAR(255) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [Folio] VARCHAR(255) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [NoCertificado] VARCHAR(25) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [LugarExpedicion] VARCHAR(10) NULL,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    -- Restricción de Integridad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    CONSTRAINT PK_ANEXO_1A_2025_1S PRIMARY KEY ([UUID])</t>
-  </si>
-  <si>
-    <t>);</t>
-  </si>
-  <si>
-    <t>Notas Arquitectónicas sobre esta tabla:</t>
-  </si>
-  <si>
-    <r>
-      <t>1. La Llave Primaria es el UUID:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A diferencia del Anexo 2B (donde inventamos el </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>HashID</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> porque un UUID se repite por cada concepto), en el Anexo 1A </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>el UUID es único</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Es la "portada" de la factura.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>2. El mismo ETL te servirá:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Cuando vayamos a cargar este archivo, usaremos la misma lógica de "Upsert" con Polars y SQLAlchemy que acabamos de diseñar. Si el archivo del SAT trae dos veces la misma cabecera por error, nuestro </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>load.py</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> simplemente insertará la primera y descartará el clon silenciosamente para no violar esta Primary Key.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>3. Manejo de Nulos:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A excepción del </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>UUID</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, todo permite </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>NULL</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Esto es vital porque, por ejemplo, una factura vigente no tendrá </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>FechaCancelacion</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, o una factura sin retenciones vendrá vacía en </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>RetenidosISR</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t>GERG_AECF_1891_Anexo2B-QA.txt</t>
-  </si>
-  <si>
-    <t>[SAT].[dbo].[AECF_1891_Anexo2B-1S2025]</t>
-  </si>
-  <si>
     <t>NOMBRE DEL CAMPO</t>
   </si>
   <si>
@@ -647,18 +331,6 @@
   </si>
   <si>
     <t>NOMBRE DE LA TABLA</t>
-  </si>
-  <si>
-    <t>Archivo origen: 449,544,219 filas</t>
-  </si>
-  <si>
-    <t>Menos 1 fila de encabezados: 449,544,218 filas de datos reales.</t>
-  </si>
-  <si>
-    <t>Diferencia: Faltan 960 registros exactos.</t>
-  </si>
-  <si>
-    <t>Tabla de Carlos en SQL: 449,543,258 registros.</t>
   </si>
   <si>
     <t>Diccionario de Datos: Anexo 3C (Cabecera de Nómina)</t>
@@ -1155,9 +827,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="171" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1166,14 +838,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -1213,19 +877,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13.5"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial Unicode MS"/>
     </font>
     <font>
       <i/>
@@ -1325,69 +976,59 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1696,13 +1337,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -1732,7 +1366,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1751,7 +1385,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1792,10 +1426,21 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
       <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1874,6 +1519,23 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -1893,27 +1555,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1929,7 +1570,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CDD1F03F-8A6A-4644-86AB-EE3BEB9D7BA0}" name="Tabla3" displayName="Tabla3" ref="A4:D32" totalsRowShown="0" headerRowDxfId="32" dataDxfId="27" headerRowBorderDxfId="34" tableBorderDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CDD1F03F-8A6A-4644-86AB-EE3BEB9D7BA0}" name="Tabla3" displayName="Tabla3" ref="A4:D32" totalsRowShown="0" headerRowDxfId="35" dataDxfId="33" headerRowBorderDxfId="34" tableBorderDxfId="32">
   <autoFilter ref="A4:D32" xr:uid="{CDD1F03F-8A6A-4644-86AB-EE3BEB9D7BA0}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{A34516A4-C803-45C1-A220-9AF4F4A18F59}" name="NOMBRE DEL CAMPO" dataDxfId="31"/>
@@ -1942,25 +1583,25 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{97A246FC-52D2-4434-AFF8-3294A7460497}" name="Tabla4" displayName="Tabla4" ref="A38:D46" totalsRowShown="0" dataDxfId="26" headerRowBorderDxfId="21" tableBorderDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{97A246FC-52D2-4434-AFF8-3294A7460497}" name="Tabla4" displayName="Tabla4" ref="A38:D46" totalsRowShown="0" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25">
   <autoFilter ref="A38:D46" xr:uid="{97A246FC-52D2-4434-AFF8-3294A7460497}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D72A1E09-2136-48A1-8F41-2EB9D14DF28D}" name="NOMBRE DEL CAMPO" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{84BDECE3-8AAC-49BF-8A04-DCBEA0FB7D08}" name="TIPO DE DATO" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{D72A1E09-2136-48A1-8F41-2EB9D14DF28D}" name="NOMBRE DEL CAMPO" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{84BDECE3-8AAC-49BF-8A04-DCBEA0FB7D08}" name="TIPO DE DATO" dataDxfId="23"/>
     <tableColumn id="3" xr3:uid="{0BC33316-7C86-47B3-B63D-A62EF998CCA5}" name="DESCRIPCIÓN" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{51F0D08A-1C39-417C-8B4E-D57E6D831E3C}" name="NUMERO DE REGISTROS" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{51F0D08A-1C39-417C-8B4E-D57E6D831E3C}" name="NUMERO DE REGISTROS" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DB3982AF-C08E-4F20-99D9-322C057C6BD6}" name="Tabla5" displayName="Tabla5" ref="A4:D25" totalsRowShown="0" headerRowBorderDxfId="19" tableBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DB3982AF-C08E-4F20-99D9-322C057C6BD6}" name="Tabla5" displayName="Tabla5" ref="A4:D25" totalsRowShown="0" headerRowBorderDxfId="20" tableBorderDxfId="19">
   <autoFilter ref="A4:D25" xr:uid="{DB3982AF-C08E-4F20-99D9-322C057C6BD6}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D8078DEB-DAF2-4C28-8C1D-B9C317BBD8A0}" name="NOMBRE DEL CAMPO" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{D8078DEB-DAF2-4C28-8C1D-B9C317BBD8A0}" name="NOMBRE DEL CAMPO" dataDxfId="18"/>
     <tableColumn id="2" xr3:uid="{631FACEB-A86F-41CD-9FF2-DFE48680F00F}" name="TIPO DE DATO" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{CEE55E1D-A47F-4993-AD91-BFCA2A837B1E}" name="DESCRIPCIÓN" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{CEE55E1D-A47F-4993-AD91-BFCA2A837B1E}" name="DESCRIPCIÓN" dataDxfId="16"/>
     <tableColumn id="4" xr3:uid="{8259B8A3-6AE0-4167-8359-A35858F5EC69}" name="NUMERO DE REGISTROS"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2337,7 +1978,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93EA6A84-B7DE-4D16-B5A1-51582A8EA647}">
   <dimension ref="A1:D46"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="63.44140625" customWidth="1"/>
     <col min="2" max="2" width="25.88671875" bestFit="1" customWidth="1"/>
@@ -2345,573 +1986,573 @@
     <col min="4" max="4" width="20.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-    </row>
-    <row r="2" spans="1:4" ht="46.8">
-      <c r="A2" s="13" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+    </row>
+    <row r="2" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B3" s="8" t="s">
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="31.2">
-      <c r="A5" s="17" t="s">
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="31.2">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="31.2">
-      <c r="A7" s="17" t="s">
+    <row r="7" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="31.2">
-      <c r="A8" s="17" t="s">
+    <row r="8" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="46.8">
-      <c r="A9" s="17" t="s">
+    <row r="9" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="31.2">
-      <c r="A10" s="17" t="s">
+    <row r="10" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="31.2">
-      <c r="A11" s="17" t="s">
+    <row r="11" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="31.2">
-      <c r="A12" s="17" t="s">
+    <row r="12" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="31.2">
-      <c r="A13" s="17" t="s">
+    <row r="13" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="18">
+      <c r="D13" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="31.2">
-      <c r="A14" s="17" t="s">
+    <row r="14" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="18">
+      <c r="D14" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="31.2">
-      <c r="A15" s="17" t="s">
+    <row r="15" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="46.8">
-      <c r="A16" s="17" t="s">
+    <row r="16" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="18">
+      <c r="D16" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="31.2">
-      <c r="A17" s="17" t="s">
+    <row r="17" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D17" s="18">
+      <c r="D17" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="31.2">
-      <c r="A18" s="17" t="s">
+    <row r="18" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="18">
+      <c r="D18" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="46.8">
-      <c r="A19" s="17" t="s">
+    <row r="19" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="D19" s="18">
+      <c r="D19" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="31.2">
-      <c r="A20" s="17" t="s">
+    <row r="20" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="D20" s="18">
+      <c r="D20" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="31.2">
-      <c r="A21" s="17" t="s">
+    <row r="21" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="D21" s="18">
+      <c r="D21" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="31.2">
-      <c r="A22" s="17" t="s">
+    <row r="22" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="18">
+      <c r="D22" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="31.2">
-      <c r="A23" s="17" t="s">
+    <row r="23" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="D23" s="18">
+      <c r="D23" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="31.2">
-      <c r="A24" s="17" t="s">
+    <row r="24" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="18">
+      <c r="D24" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="31.2">
-      <c r="A25" s="17" t="s">
+    <row r="25" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="C25" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="D25" s="18">
+      <c r="D25" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="46.8">
-      <c r="A26" s="17" t="s">
+    <row r="26" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="D26" s="18">
+      <c r="D26" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="46.8">
-      <c r="A27" s="17" t="s">
+    <row r="27" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="C27" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="D27" s="18">
+      <c r="D27" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="31.2">
-      <c r="A28" s="17" t="s">
+    <row r="28" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="C28" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="18">
+      <c r="D28" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="31.2">
-      <c r="A29" s="17" t="s">
+    <row r="29" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="D29" s="18">
+      <c r="D29" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="31.2">
-      <c r="A30" s="17" t="s">
+    <row r="30" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A30" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B30" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="D30" s="18">
+      <c r="D30" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="31.2">
-      <c r="A31" s="17" t="s">
+    <row r="31" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="B31" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="C31" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="D31" s="18">
+      <c r="D31" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="31.2">
-      <c r="A32" s="17" t="s">
+    <row r="32" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B32" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C32" s="17" t="s">
+      <c r="C32" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="D32" s="18">
+      <c r="D32" s="12">
         <v>203304109</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="15.6">
-      <c r="A35" s="11" t="s">
+    <row r="35" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B35" s="12"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="12"/>
-    </row>
-    <row r="36" spans="1:4" ht="46.8">
-      <c r="A36" s="13" t="s">
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+    </row>
+    <row r="36" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-    </row>
-    <row r="37" spans="1:4" ht="14.4" customHeight="1">
-      <c r="A37" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B37" s="19" t="s">
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+    </row>
+    <row r="37" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B37" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="C38" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="D38" s="15" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="31.2">
-      <c r="A39" s="21" t="s">
+      <c r="C37" s="19"/>
+      <c r="D37" s="19"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B39" s="21" t="s">
+      <c r="B39" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="21" t="s">
+      <c r="C39" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D39" s="16"/>
-    </row>
-    <row r="40" spans="1:4" ht="31.2">
-      <c r="A40" s="21" t="s">
+      <c r="D39" s="10"/>
+    </row>
+    <row r="40" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A40" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="B40" s="21" t="s">
+      <c r="B40" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="C40" s="21" t="s">
+      <c r="C40" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="D40" s="16"/>
-    </row>
-    <row r="41" spans="1:4" ht="46.8">
-      <c r="A41" s="21" t="s">
+      <c r="D40" s="10"/>
+    </row>
+    <row r="41" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A41" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="B41" s="21" t="s">
+      <c r="B41" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="C41" s="21" t="s">
+      <c r="C41" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="D41" s="16"/>
-    </row>
-    <row r="42" spans="1:4" ht="31.2">
-      <c r="A42" s="21" t="s">
+      <c r="D41" s="10"/>
+    </row>
+    <row r="42" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A42" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B42" s="21" t="s">
+      <c r="B42" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C42" s="21" t="s">
+      <c r="C42" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="D42" s="16"/>
-    </row>
-    <row r="43" spans="1:4" ht="31.2">
-      <c r="A43" s="21" t="s">
+      <c r="D42" s="10"/>
+    </row>
+    <row r="43" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A43" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="B43" s="21" t="s">
+      <c r="B43" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="C43" s="21" t="s">
+      <c r="C43" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="D43" s="16"/>
-    </row>
-    <row r="44" spans="1:4" ht="46.8">
-      <c r="A44" s="21" t="s">
+      <c r="D43" s="10"/>
+    </row>
+    <row r="44" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A44" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="B44" s="21" t="s">
+      <c r="B44" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="C44" s="21" t="s">
+      <c r="C44" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="D44" s="16"/>
-    </row>
-    <row r="45" spans="1:4" ht="46.8">
-      <c r="A45" s="21" t="s">
+      <c r="D44" s="10"/>
+    </row>
+    <row r="45" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A45" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="B45" s="21" t="s">
+      <c r="B45" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C45" s="21" t="s">
+      <c r="C45" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="D45" s="16"/>
-    </row>
-    <row r="46" spans="1:4" ht="46.8">
-      <c r="A46" s="21" t="s">
+      <c r="D45" s="10"/>
+    </row>
+    <row r="46" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="B46" s="21" t="s">
+      <c r="B46" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C46" s="21" t="s">
+      <c r="C46" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="D46" s="16"/>
+      <c r="D46" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2929,49 +2570,49 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F218ABF-3A67-4416-99D5-21948A961EB5}">
   <dimension ref="A1:D77"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="67.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="76.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="1" max="1" width="170.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="119.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6">
+    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.6">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="27.6">
-      <c r="A3" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B3" s="8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-    </row>
-    <row r="4" spans="1:4" ht="27.6">
-      <c r="A4" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="D4" s="23" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.6">
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
@@ -2979,219 +2620,219 @@
         <v>30</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>155</v>
+        <v>101</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.6">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>155</v>
+        <v>101</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.6">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>158</v>
+        <v>104</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>57</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.6">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>191</v>
+        <v>137</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>160</v>
+        <v>106</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.6">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>162</v>
+        <v>108</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.6">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>164</v>
+        <v>110</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.6">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>166</v>
+        <v>112</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.6">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>168</v>
+        <v>114</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.6">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>192</v>
+        <v>138</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.6">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>171</v>
+        <v>117</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.6">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>173</v>
+        <v>119</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.6">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>175</v>
+        <v>121</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>176</v>
+        <v>122</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.6">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>193</v>
+        <v>139</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>178</v>
+        <v>124</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="15.6">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>180</v>
+        <v>126</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>59</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="15.6">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>182</v>
+        <v>128</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>160</v>
+        <v>106</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15.6">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>194</v>
+        <v>140</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>64</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="15.6">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>185</v>
+        <v>131</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>83</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="15.6">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>195</v>
+        <v>141</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>61</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15.6">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>196</v>
+        <v>142</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>188</v>
+        <v>134</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="15.6">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>27</v>
       </c>
@@ -3199,44 +2840,44 @@
         <v>32</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="15.6">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15.6">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B30" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B30" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="B31" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="C31" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="D31" s="23" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="15.6">
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>0</v>
       </c>
@@ -3244,99 +2885,99 @@
         <v>30</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="15.6">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>200</v>
+        <v>146</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>155</v>
+        <v>101</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="15.6">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>202</v>
+        <v>148</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>64</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="15.6">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>204</v>
+        <v>150</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>59</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="15.6">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>206</v>
+        <v>152</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>61</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="15.6">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>208</v>
+        <v>154</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="15.6">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="15.6">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="A42" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B42" s="8" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B42" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="B43" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="C43" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="D43" s="23" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="15.6">
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B43" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D43" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>0</v>
       </c>
@@ -3344,306 +2985,306 @@
         <v>30</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="15.6">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>200</v>
+        <v>146</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>155</v>
+        <v>101</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="15.6">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>212</v>
+        <v>158</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>64</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="15.6">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>214</v>
+        <v>160</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>59</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="15.6">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>216</v>
+        <v>162</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>61</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="15.6">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>218</v>
+        <v>164</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="15.6">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="15.6">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4">
-      <c r="A54" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B54" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B54" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="C54" s="9"/>
-      <c r="D54" s="9"/>
-    </row>
-    <row r="55" spans="1:4">
-      <c r="A55" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="B55" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="C55" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="D55" s="23" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="15.6">
+      <c r="C54" s="17"/>
+      <c r="D54" s="17"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B55" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C55" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D55" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>222</v>
+        <v>168</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="15.6">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>224</v>
+        <v>170</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="15.6">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>226</v>
+        <v>172</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="15.6">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>228</v>
+        <v>174</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="15.6">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>230</v>
+        <v>176</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="15.6">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
-        <v>232</v>
+        <v>178</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="15.6">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>234</v>
+        <v>180</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>235</v>
+        <v>181</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="15.6">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>237</v>
+        <v>183</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="15.6">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>239</v>
+        <v>185</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" ht="15.6">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" ht="15.6">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4">
-      <c r="A69" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B69" s="8" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="C69" s="9"/>
-      <c r="D69" s="9"/>
-    </row>
-    <row r="70" spans="1:4">
-      <c r="A70" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="B70" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="C70" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="D70" s="23" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" ht="15.6">
+      <c r="C69" s="17"/>
+      <c r="D69" s="17"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A70" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B70" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C70" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D70" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
-        <v>222</v>
+        <v>168</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" ht="15.6">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
-        <v>243</v>
+        <v>189</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>235</v>
+        <v>181</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" ht="15.6">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
-        <v>245</v>
+        <v>191</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>64</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" ht="15.6">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
-        <v>247</v>
+        <v>193</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" ht="15.6">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
-        <v>249</v>
+        <v>195</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" ht="15.6">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
-        <v>251</v>
+        <v>197</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" ht="15.6">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
-        <v>253</v>
+        <v>199</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>254</v>
+        <v>200</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>255</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -3663,302 +3304,4 @@
     <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AEF4A3A-B5CC-45B7-B335-8FEBCB625601}">
-  <dimension ref="A1:I47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" ht="18">
-      <c r="A1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E1" t="s">
-        <v>96</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B2" s="4">
-        <v>449544219</v>
-      </c>
-      <c r="E2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I2" s="6"/>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B3" s="4">
-        <v>449544219</v>
-      </c>
-      <c r="E3" t="s">
-        <v>98</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" t="s">
-        <v>142</v>
-      </c>
-      <c r="B4" s="4">
-        <v>449543258</v>
-      </c>
-      <c r="E4" t="s">
-        <v>99</v>
-      </c>
-      <c r="I4" s="6"/>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="E5" t="s">
-        <v>100</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="E6" t="s">
-        <v>101</v>
-      </c>
-      <c r="I6" s="6"/>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="E7" t="s">
-        <v>102</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="E8" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="E9" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="E10" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="6"/>
-      <c r="E11" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="E12" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="6"/>
-      <c r="E13" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="7"/>
-      <c r="E14" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="E15" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="E16" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="17" spans="5:5">
-      <c r="E17" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="18" spans="5:5">
-      <c r="E18" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="19" spans="5:5">
-      <c r="E19" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="20" spans="5:5">
-      <c r="E20" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="21" spans="5:5">
-      <c r="E21" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="22" spans="5:5">
-      <c r="E22" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="23" spans="5:5">
-      <c r="E23" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="24" spans="5:5">
-      <c r="E24" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="25" spans="5:5">
-      <c r="E25" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="26" spans="5:5">
-      <c r="E26" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="27" spans="5:5">
-      <c r="E27" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="28" spans="5:5">
-      <c r="E28" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="29" spans="5:5">
-      <c r="E29" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="30" spans="5:5">
-      <c r="E30" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="31" spans="5:5">
-      <c r="E31" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="32" spans="5:5">
-      <c r="E32" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="33" spans="5:5">
-      <c r="E33" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="34" spans="5:5">
-      <c r="E34" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="35" spans="5:5">
-      <c r="E35" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="36" spans="5:5">
-      <c r="E36" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="37" spans="5:5">
-      <c r="E37" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="38" spans="5:5">
-      <c r="E38" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="39" spans="5:5">
-      <c r="E39" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="40" spans="5:5">
-      <c r="E40" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="41" spans="5:5">
-      <c r="E41" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="42" spans="5:5">
-      <c r="E42" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="43" spans="5:5">
-      <c r="E43" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="45" spans="5:5">
-      <c r="E45" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="46" spans="5:5">
-      <c r="E46" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="47" spans="5:5">
-      <c r="E47" t="s">
-        <v>136</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>